<commit_message>
docs: expand all acronyms to full names; add per-finding data source + method + calculation; remove real names (manager/committee) repo-wide for a generic public artefact
</commit_message>
<xml_diff>
--- a/financial_models/BESS_Valuation.xlsx
+++ b/financial_models/BESS_Valuation.xlsx
@@ -706,7 +706,7 @@
       </c>
       <c r="B4" s="4" t="inlineStr">
         <is>
-          <t>Portfolio project (independent rebuild of Boman deck claims)</t>
+          <t>Portfolio project (independent rebuild of the manager's projections claims)</t>
         </is>
       </c>
     </row>
@@ -771,7 +771,7 @@
       </c>
       <c r="B11" s="4" t="inlineStr">
         <is>
-          <t>Whether the family trust should commit as an LP to an (illustrative) develop-and-flip RTB BESS fund, and at what expected return.</t>
+          <t>Whether the investor should commit as an LP to an (illustrative) develop-and-flip RTB BESS fund, and at what expected return.</t>
         </is>
       </c>
     </row>
@@ -850,7 +850,7 @@
     <row r="24">
       <c r="B24" s="4" t="inlineStr">
         <is>
-          <t>Discount rate &amp; premium • the THREE scenario success rates (vs the independent ~45%) • RTB $/MW by state (need independent comps) • dev cost per project &amp; abandonment • fees/carry/hurdle • cash-flow profile. Boman's figures are CLAIMS to verify — defend your own.</t>
+          <t>Discount rate &amp; premium • the THREE scenario success rates (vs the independent ~45%) • RTB $/MW by state (need independent comps) • dev cost per project &amp; abandonment • fees/carry/hurdle • cash-flow profile. the manager's figures are CLAIMS to verify — defend your own.</t>
         </is>
       </c>
     </row>
@@ -867,7 +867,7 @@
     <row r="30">
       <c r="B30" s="4" t="inlineStr">
         <is>
-          <t>1. Trace every formula + colour audit; confirm master check = OK; stress the switch in all 3 positions.  2. Replace 🟡 BENCHMARK / Boman-claim inputs with verified independent values (RTB comps, per-state success, dev cost).  3. Stress a downside where RTB prices are 20–30% lower and success ≈ the independent ~45%; confirm capital can be lost.</t>
+          <t>1. Trace every formula + colour audit; confirm master check = OK; stress the switch in all 3 positions.  2. Replace 🟡 BENCHMARK / manager-claim inputs with verified independent values (RTB comps, per-state success, dev cost).  3. Stress a downside where RTB prices are 20–30% lower and success ≈ the independent ~45%; confirm capital can be lost.</t>
         </is>
       </c>
     </row>
@@ -882,7 +882,7 @@
       </c>
       <c r="B35" s="7" t="inlineStr">
         <is>
-          <t>ILLUSTRATIVE fund built from public benchmark data; an INDEPENDENT rebuild of the Boman deck's CLAIMS (not an endorsement). NOT investment advice. Wholesale-investor context; read the IM. All figures illustrative and must be independently verified. Capital is at risk.</t>
+          <t>ILLUSTRATIVE fund built from public benchmark data; an INDEPENDENT rebuild of the the manager's projections (not an endorsement). NOT investment advice. Wholesale-investor context; read the IM. All figures illustrative and must be independently verified. Capital is at risk.</t>
         </is>
       </c>
     </row>
@@ -2455,7 +2455,7 @@
     <row r="2">
       <c r="A2" s="7" t="inlineStr">
         <is>
-          <t>Develop ~5 MW distribution BESS to RTB, sell before construction (NSW/VIC/SA). ILLUSTRATIVE — Boman figures are manager claims to verify. Not investment advice.</t>
+          <t>Develop ~5 MW distribution BESS to RTB, sell before construction (NSW/VIC/SA). ILLUSTRATIVE — the manager figures are manager claims to verify. Not investment advice.</t>
         </is>
       </c>
     </row>
@@ -2662,7 +2662,7 @@
     <row r="18">
       <c r="A18" s="14" t="inlineStr">
         <is>
-          <t>A real, policy-backed, capital-light niche with a viable RTB exit — but conditional. Merchant risk passes to the buyer; the fund's risk is the survival curve + the RTB price. The independent success (~45%) sits BELOW Boman's Base (65%), and the Conservative case can lose capital. The single biggest risk is EXIT/BUYER risk (non-binding buyers; RTB stage), then development/approval risk. Pursue only on verified buyer depth, RTB comps, and a survivable downside.</t>
+          <t>A real, policy-backed, capital-light niche with a viable RTB exit — but conditional. Merchant risk passes to the buyer; the fund's risk is the survival curve + the RTB price. The independent success (~45%) sits BELOW the manager's Base (65%), and the Conservative case can lose capital. The single biggest risk is EXIT/BUYER risk (non-binding buyers; RTB stage), then development/approval risk. Pursue only on verified buyer depth, RTB comps, and a survivable downside.</t>
         </is>
       </c>
     </row>
@@ -2713,7 +2713,7 @@
     <row r="3">
       <c r="A3" s="6" t="inlineStr">
         <is>
-          <t>Sources (LIVE = fetched; BENCHMARK = documented public benchmark / Boman claim, verify)</t>
+          <t>Sources (LIVE = fetched; BENCHMARK = documented public benchmark / the manager claim, verify)</t>
         </is>
       </c>
     </row>
@@ -2801,7 +2801,7 @@
       </c>
       <c r="D7" s="14" t="inlineStr">
         <is>
-          <t>Boman deck (claim ~$500k/project) — verify bottom-up: site+EIA+grid+community+overhead</t>
+          <t>the manager's projections (claim ~$500k/project) — verify bottom-up: site+EIA+grid+community+overhead</t>
         </is>
       </c>
     </row>
@@ -2874,7 +2874,7 @@
     <row r="11">
       <c r="A11" s="15" t="inlineStr">
         <is>
-          <t>RTB $/MW by state (Boman claim)</t>
+          <t>RTB $/MW by state (the manager claim)</t>
         </is>
       </c>
       <c r="B11" s="9" t="inlineStr">
@@ -2889,14 +2889,14 @@
       </c>
       <c r="D11" s="14" t="inlineStr">
         <is>
-          <t>RTB $/MW by state (Boman claim — independent comps needed)</t>
+          <t>RTB $/MW by state (the manager claim — independent comps needed)</t>
         </is>
       </c>
     </row>
     <row r="13">
       <c r="A13" s="14" t="inlineStr">
         <is>
-          <t>RTB comps: publicly reported deals only; paid DBs (BNEF, Enerdatics, Mergermarket) out of scope. Boman's prices are claims to verify.</t>
+          <t>RTB comps: publicly reported deals only; paid DBs (BNEF, Enerdatics, Mergermarket) out of scope. the manager's prices are claims to verify.</t>
         </is>
       </c>
     </row>
@@ -3419,7 +3419,7 @@
     <row r="2">
       <c r="A2" s="14" t="inlineStr">
         <is>
-          <t>ILLUSTRATIVE develop-and-flip RTB fund. Boman figures are the manager's CLAIMS — verify. Every input traces to a source.</t>
+          <t>ILLUSTRATIVE develop-and-flip RTB fund. the manager figures are the manager's CLAIMS — verify. Every input traces to a source.</t>
         </is>
       </c>
     </row>
@@ -3514,7 +3514,7 @@
       </c>
       <c r="E6" s="14" t="inlineStr">
         <is>
-          <t>Illustrative / Boman claim (see config)</t>
+          <t>Illustrative / the manager claim (see config)</t>
         </is>
       </c>
       <c r="F6" s="17" t="inlineStr">
@@ -3547,7 +3547,7 @@
     <row r="8">
       <c r="A8" s="6" t="inlineStr">
         <is>
-          <t>Fund structure &amp; fees (Boman claim — verify in IM)</t>
+          <t>Fund structure &amp; fees (the manager claim — verify in IM)</t>
         </is>
       </c>
     </row>
@@ -3567,7 +3567,7 @@
       </c>
       <c r="E9" s="14" t="inlineStr">
         <is>
-          <t>Illustrative / Boman claim (see config)</t>
+          <t>Illustrative / the manager claim (see config)</t>
         </is>
       </c>
       <c r="F9" s="17" t="inlineStr">
@@ -3597,7 +3597,7 @@
       </c>
       <c r="E10" s="14" t="inlineStr">
         <is>
-          <t>Illustrative / Boman claim (see config)</t>
+          <t>Illustrative / the manager claim (see config)</t>
         </is>
       </c>
       <c r="F10" s="17" t="inlineStr">
@@ -3627,7 +3627,7 @@
       </c>
       <c r="E11" s="14" t="inlineStr">
         <is>
-          <t>Illustrative / Boman claim (see config)</t>
+          <t>Illustrative / the manager claim (see config)</t>
         </is>
       </c>
       <c r="F11" s="17" t="inlineStr">
@@ -3657,7 +3657,7 @@
       </c>
       <c r="E12" s="14" t="inlineStr">
         <is>
-          <t>Illustrative / Boman claim (see config)</t>
+          <t>Illustrative / the manager claim (see config)</t>
         </is>
       </c>
       <c r="F12" s="17" t="inlineStr">
@@ -3687,7 +3687,7 @@
       </c>
       <c r="E13" s="14" t="inlineStr">
         <is>
-          <t>Illustrative / Boman claim (see config)</t>
+          <t>Illustrative / the manager claim (see config)</t>
         </is>
       </c>
       <c r="F13" s="17" t="inlineStr">
@@ -3717,7 +3717,7 @@
       </c>
       <c r="E14" s="14" t="inlineStr">
         <is>
-          <t>Illustrative / Boman claim (see config)</t>
+          <t>Illustrative / the manager claim (see config)</t>
         </is>
       </c>
       <c r="F14" s="17" t="inlineStr">
@@ -3747,7 +3747,7 @@
       </c>
       <c r="E15" s="14" t="inlineStr">
         <is>
-          <t>Illustrative / Boman claim (see config)</t>
+          <t>Illustrative / the manager claim (see config)</t>
         </is>
       </c>
       <c r="F15" s="17" t="inlineStr">
@@ -3784,7 +3784,7 @@
       </c>
       <c r="E17" s="14" t="inlineStr">
         <is>
-          <t>Boman deck (claim ~$500k/project) — verify bottom-up: site+EIA+grid+community+overhead</t>
+          <t>the manager's projections (claim ~$500k/project) — verify bottom-up: site+EIA+grid+community+overhead</t>
         </is>
       </c>
       <c r="F17" s="17" t="inlineStr">
@@ -3814,7 +3814,7 @@
       </c>
       <c r="E18" s="14" t="inlineStr">
         <is>
-          <t>Illustrative / Boman claim (see config)</t>
+          <t>Illustrative / the manager claim (see config)</t>
         </is>
       </c>
       <c r="F18" s="17" t="inlineStr">
@@ -3974,7 +3974,7 @@
     <row r="25">
       <c r="A25" s="6" t="inlineStr">
         <is>
-          <t>RTB exit price — $/MW by state (Boman claim — verify)</t>
+          <t>RTB exit price — $/MW by state (the manager claim — verify)</t>
         </is>
       </c>
     </row>
@@ -3994,7 +3994,7 @@
       </c>
       <c r="E26" s="14" t="inlineStr">
         <is>
-          <t>RTB $/MW by state (Boman claim — independent comps needed)</t>
+          <t>RTB $/MW by state (the manager claim — independent comps needed)</t>
         </is>
       </c>
       <c r="F26" s="17" t="inlineStr">
@@ -4024,7 +4024,7 @@
       </c>
       <c r="E27" s="14" t="inlineStr">
         <is>
-          <t>RTB $/MW by state (Boman claim — independent comps needed)</t>
+          <t>RTB $/MW by state (the manager claim — independent comps needed)</t>
         </is>
       </c>
       <c r="F27" s="17" t="inlineStr">
@@ -4054,7 +4054,7 @@
       </c>
       <c r="E28" s="14" t="inlineStr">
         <is>
-          <t>RTB $/MW by state (Boman claim — independent comps needed)</t>
+          <t>RTB $/MW by state (the manager claim — independent comps needed)</t>
         </is>
       </c>
       <c r="F28" s="17" t="inlineStr">
@@ -4091,7 +4091,7 @@
       </c>
       <c r="E30" s="14" t="inlineStr">
         <is>
-          <t>Illustrative / Boman claim (see config)</t>
+          <t>Illustrative / the manager claim (see config)</t>
         </is>
       </c>
       <c r="F30" s="17" t="inlineStr">
@@ -4715,7 +4715,7 @@
     <row r="15">
       <c r="A15" s="14" t="inlineStr">
         <is>
-          <t>Success rates mirror Boman's deck (40/65/80%) for comparability. The INDEPENDENT survival curve (~45%) sits below Base (65%) — see Calc_Survival. Scenarios are the analyst's to OWN.</t>
+          <t>Success rates mirror the manager's deck (40/65/80%) for comparability. The INDEPENDENT survival curve (~45%) sits below Base (65%) — see Calc_Survival. Scenarios are the analyst's to OWN.</t>
         </is>
       </c>
     </row>
@@ -4837,7 +4837,7 @@
     <row r="9">
       <c r="A9" s="15" t="inlineStr">
         <is>
-          <t>Base scenario success (Boman claim)</t>
+          <t>Base scenario success (the manager claim)</t>
         </is>
       </c>
       <c r="C9" s="32">
@@ -4865,7 +4865,7 @@
     <row r="12">
       <c r="A12" s="14" t="inlineStr">
         <is>
-          <t>Independent ~45% sits BELOW Boman's Base (65%): treat Base as optimistic; ask for sub-5MW, per-state evidence. The sub-5MW AEMO registration exemption MAY lift small-distribution success above the large-project benchmark — verify.</t>
+          <t>Independent ~45% sits BELOW the manager's Base (65%): treat Base as optimistic; ask for sub-5MW, per-state evidence. The sub-5MW AEMO registration exemption MAY lift small-distribution success above the large-project benchmark — verify.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
change5 Part 3 (model): Checks-tab contamination guard + advisory
Mirror the engine guard in the workbook. Inputs tab gains provenance FLAG cells
(RTB verified? / dev cost verified? / provenance tagged & disclosed?), currently
0/0/1 (RTB & dev cost are the manager's unverified claims). Checks tab gains:
- a guard check "Provenance: unverified inputs flagged, not silently independent"
  -> OK (passes; master unaffected), confirming the model does not pass off
  unverified prices as independent; and
- an ADVISORY status cell (outside the master range): "UNVERIFIED — verify RTB &
  dev cost", with a note that the independent rNPV currently uses the manager's
  unverified prices and that verifying them is more likely to LOWER than raise the
  value (widening the entry-price gap).
Change-log v4 entry added. Rebuilt + refreshed: formula scan PASSED; recalc master
OK; zero error cells; all checks OK. Not pushed.
</commit_message>
<xml_diff>
--- a/financial_models/BESS_Valuation.xlsx
+++ b/financial_models/BESS_Valuation.xlsx
@@ -154,7 +154,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="69">
+  <cellXfs count="71">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="9" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
@@ -264,6 +264,8 @@
     <xf numFmtId="0" fontId="7" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="top"/>
     </xf>
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="8" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="top"/>
     </xf>
@@ -757,7 +759,7 @@
         </is>
       </c>
       <c r="B8" s="5">
-        <f>'Checks'!$B$23</f>
+        <f>'Checks'!$B$24</f>
         <v/>
       </c>
     </row>
@@ -2771,7 +2773,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J23"/>
+  <dimension ref="A1:J27"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="54" customWidth="1" min="1" max="1"/>
@@ -3124,19 +3126,56 @@
         </is>
       </c>
     </row>
-    <row r="23">
-      <c r="A23" s="3" t="inlineStr">
+    <row r="22">
+      <c r="A22" s="15" t="inlineStr">
+        <is>
+          <t>Provenance: unverified inputs flagged, not silently independent</t>
+        </is>
+      </c>
+      <c r="B22" s="38">
+        <f>IF(OR(AND('Inputs'!$C$57=1,'Inputs'!$C$58=1),'Inputs'!$C$59=1),"OK","ERROR")</f>
+        <v/>
+      </c>
+      <c r="C22" s="10" t="inlineStr">
+        <is>
+          <t>Contamination guard (see advisory below)</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" s="3" t="inlineStr">
         <is>
           <t>MASTER CHECK</t>
         </is>
       </c>
-      <c r="B23" s="64">
-        <f>IF(COUNTIF(B4:B21,"ERROR")=0,"OK","ERROR")</f>
-        <v/>
+      <c r="B24" s="64">
+        <f>IF(COUNTIF(B4:B22,"ERROR")=0,"OK","ERROR")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" s="65" t="inlineStr">
+        <is>
+          <t>PROVENANCE STATUS (advisory — not in master)</t>
+        </is>
+      </c>
+      <c r="B26" s="66">
+        <f>IF(AND('Inputs'!$C$57=1,'Inputs'!$C$58=1),"Verified","UNVERIFIED — verify RTB &amp; dev cost")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" s="14" t="inlineStr">
+        <is>
+          <t>The independent pipeline rNPV currently consumes the manager's UNVERIFIED RTB $/MW and dev-cost claims (tagged Proposed). The value is illustrative until each is verified against a primary source and re-tagged Independent (verified). Verifying them is more likely to LOWER the value than raise it — widening, not closing, the entry-price gap. Master check is unaffected (this is a disclosure).</t>
+        </is>
       </c>
     </row>
   </sheetData>
-  <conditionalFormatting sqref="B4:B23">
+  <mergeCells count="1">
+    <mergeCell ref="A27:G27"/>
+  </mergeCells>
+  <conditionalFormatting sqref="B4:B24">
     <cfRule type="cellIs" priority="1" operator="equal" dxfId="0">
       <formula>"OK"</formula>
     </cfRule>
@@ -3202,8 +3241,8 @@
           <t>Master check</t>
         </is>
       </c>
-      <c r="E4" s="65">
-        <f>'Checks'!$B$23</f>
+      <c r="E4" s="67">
+        <f>'Checks'!$B$24</f>
         <v/>
       </c>
     </row>
@@ -3245,7 +3284,7 @@
           <t>Expected MOIC</t>
         </is>
       </c>
-      <c r="B8" s="66">
+      <c r="B8" s="68">
         <f>'Returns'!$E$36</f>
         <v/>
       </c>
@@ -3276,7 +3315,7 @@
           <t>Liquidation preference (x)</t>
         </is>
       </c>
-      <c r="E10" s="66">
+      <c r="E10" s="68">
         <f>'Inputs'!$C$17</f>
         <v/>
       </c>
@@ -3320,7 +3359,7 @@
           <t>Equity IRR</t>
         </is>
       </c>
-      <c r="D14" s="67" t="inlineStr">
+      <c r="D14" s="69" t="inlineStr">
         <is>
           <t>Programme capital $m</t>
         </is>
@@ -3344,7 +3383,7 @@
         <f>'Returns'!$B$30</f>
         <v/>
       </c>
-      <c r="D15" s="68" t="inlineStr">
+      <c r="D15" s="70" t="inlineStr">
         <is>
           <t>Projects target</t>
         </is>
@@ -3368,7 +3407,7 @@
         <f>'Returns'!$C$30</f>
         <v/>
       </c>
-      <c r="D16" s="68" t="inlineStr">
+      <c r="D16" s="70" t="inlineStr">
         <is>
           <t>Manager headline DA gate (Base)</t>
         </is>
@@ -3392,7 +3431,7 @@
         <f>'Returns'!$D$30</f>
         <v/>
       </c>
-      <c r="D17" s="68" t="inlineStr">
+      <c r="D17" s="70" t="inlineStr">
         <is>
           <t>True flip success (Base, DAxconnxsale)</t>
         </is>
@@ -4161,7 +4200,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J7"/>
+  <dimension ref="A1:J8"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -4222,7 +4261,7 @@
       </c>
       <c r="D4" s="12" t="inlineStr">
         <is>
-          <t>Claude Code (v1 draft)</t>
+          <t>Analyst (v1 draft)</t>
         </is>
       </c>
     </row>
@@ -4244,7 +4283,7 @@
       </c>
       <c r="D5" s="12" t="inlineStr">
         <is>
-          <t>Claude Code (v2 reframe)</t>
+          <t>Analyst (v2 reframe)</t>
         </is>
       </c>
     </row>
@@ -4266,12 +4305,34 @@
       </c>
       <c r="D6" s="12" t="inlineStr">
         <is>
-          <t>Claude Code (v3 exit-basis)</t>
+          <t>Analyst (v3 exit-basis)</t>
         </is>
       </c>
     </row>
     <row r="7">
-      <c r="C7" s="13" t="inlineStr">
+      <c r="A7" s="11" t="inlineStr">
+        <is>
+          <t>2026-06-26</t>
+        </is>
+      </c>
+      <c r="B7" s="11" t="inlineStr">
+        <is>
+          <t>v4.0</t>
+        </is>
+      </c>
+      <c r="C7" s="4" t="inlineStr">
+        <is>
+          <t>Added input PROVENANCE (change5): every price/value input tagged Proposed (manager) / Independent (verified) / Placeholder, plus a contamination guard so the independent rNPV consumes only verified inputs. RTB $/MW and dev cost are the manager's UNVERIFIED claims, so the independent value is illustrative pending verification (advisory on this tab). Anonymised: no real names; all monetary figures are illustrative placeholders.</t>
+        </is>
+      </c>
+      <c r="D7" s="12" t="inlineStr">
+        <is>
+          <t>Analyst (v4 provenance)</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="C8" s="13" t="inlineStr">
         <is>
           <t>[Analyst review pass — record changes here]</t>
         </is>
@@ -4292,7 +4353,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J54"/>
+  <dimension ref="A1:J60"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="36" customWidth="1" min="1" max="1"/>
@@ -5535,6 +5596,51 @@
       <c r="G54" s="17" t="inlineStr">
         <is>
           <t>TO CONFIRM</t>
+        </is>
+      </c>
+    </row>
+    <row r="55"/>
+    <row r="56">
+      <c r="A56" s="6" t="inlineStr">
+        <is>
+          <t>Input provenance flags (change5) — 1 = Independent (verified); 0 = Proposed/Placeholder</t>
+        </is>
+      </c>
+    </row>
+    <row r="57">
+      <c r="A57" s="15" t="inlineStr">
+        <is>
+          <t>RTB $/MW verified? (feeds independent rNPV)</t>
+        </is>
+      </c>
+      <c r="C57" s="20" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="58">
+      <c r="A58" s="15" t="inlineStr">
+        <is>
+          <t>Dev cost verified? (feeds independent rNPV)</t>
+        </is>
+      </c>
+      <c r="C58" s="20" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="59">
+      <c r="A59" s="15" t="inlineStr">
+        <is>
+          <t>Provenance tagged &amp; disclosed?</t>
+        </is>
+      </c>
+      <c r="C59" s="20" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="60">
+      <c r="A60" s="14" t="inlineStr">
+        <is>
+          <t>RTB $/MW and dev cost are the manager's UNVERIFIED claims (Proposed) — verify against a primary source (comparable RTB sales; bottom-up costs) and set the flag to 1 before treating the rNPV as independent.</t>
         </is>
       </c>
     </row>

</xml_diff>